<commit_message>
Fix: template template_format_A_triangle_cumule.xlsx — en-têtes ligne 1 (pandas lisible)
</commit_message>
<xml_diff>
--- a/direction_non_vie/services/templates/template_format_A_triangle_cumule.xlsx
+++ b/direction_non_vie/services/templates/template_format_A_triangle_cumule.xlsx
@@ -29,20 +29,19 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00C9A84C"/>
-      <sz val="13"/>
+      <color rgb="000F2E52"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="000F2E52"/>
-      <sz val="11"/>
+      <color rgb="00C9A84C"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00F0F4F8"/>
-      <sz val="11"/>
+      <color rgb="000F2E52"/>
+      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -53,7 +52,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000F2E52"/>
-      <sz val="14"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -70,12 +69,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000F2E52"/>
+        <fgColor rgb="00C9A84C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C9A84C"/>
+        <fgColor rgb="000F2E52"/>
       </patternFill>
     </fill>
     <fill>
@@ -99,20 +98,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00FFFFFF"/>
-      </left>
-      <right style="thin">
-        <color rgb="00FFFFFF"/>
-      </right>
-      <top style="thin">
-        <color rgb="00FFFFFF"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00FFFFFF"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="00243F6A"/>
       </left>
       <right style="thin">
@@ -125,13 +110,27 @@
         <color rgb="00243F6A"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="000A1F38"/>
+      </left>
+      <right style="thin">
+        <color rgb="000A1F38"/>
+      </right>
+      <top style="thin">
+        <color rgb="000A1F38"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="000A1F38"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -140,12 +139,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -512,7 +510,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -528,266 +526,260 @@
     <col width="13" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1" ht="22" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ActuarIA — Format A : Triangle Cumulé (Paiements)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Survenance \ Dev.</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 1</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 2</t>
-        </is>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 3</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 4</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 5</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 6</t>
-        </is>
-      </c>
-      <c r="H2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 7</t>
-        </is>
-      </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 8</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 9</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>Dev. 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="2" t="n">
+          <t>Survenance</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="I1" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="J1" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K1" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="n">
         <v>1981</v>
       </c>
+      <c r="B2" s="4" t="n">
+        <v>357848</v>
+      </c>
+      <c r="C2" s="4" t="n">
+        <v>1124788</v>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>1735330</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>2218270</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>2745596</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>3319994</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>3466336</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>3606286</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>3833515</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>3901463</v>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>1982</v>
+      </c>
       <c r="B3" s="4" t="n">
-        <v>357848</v>
+        <v>352118</v>
       </c>
       <c r="C3" s="4" t="n">
-        <v>1124788</v>
+        <v>1236139</v>
       </c>
       <c r="D3" s="4" t="n">
-        <v>1735330</v>
+        <v>2170106</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>2218270</v>
+        <v>3353322</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>2745596</v>
+        <v>3799067</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>3319994</v>
+        <v>4120063</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>3466336</v>
+        <v>4647867</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>3606286</v>
+        <v>4914039</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>3833515</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>3901463</v>
-      </c>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="2" t="n">
-        <v>1982</v>
+        <v>5339085</v>
+      </c>
+      <c r="K3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>1983</v>
       </c>
       <c r="B4" s="4" t="n">
-        <v>352118</v>
+        <v>290507</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>1236139</v>
+        <v>1292306</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>2170106</v>
+        <v>2218525</v>
       </c>
       <c r="E4" s="4" t="n">
-        <v>3353322</v>
+        <v>3235179</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>3799067</v>
+        <v>3985995</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>4120063</v>
+        <v>4132918</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>4647867</v>
+        <v>4628910</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>4914039</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>5339085</v>
-      </c>
+        <v>4909315</v>
+      </c>
+      <c r="J4" s="5" t="n"/>
       <c r="K4" s="5" t="n"/>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="2" t="n">
-        <v>1983</v>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>1984</v>
       </c>
       <c r="B5" s="4" t="n">
-        <v>290507</v>
+        <v>310608</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>1292306</v>
+        <v>1418858</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>2218525</v>
+        <v>2195047</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>3235179</v>
+        <v>3757447</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>3985995</v>
+        <v>4029929</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>4132918</v>
+        <v>4381982</v>
       </c>
       <c r="H5" s="4" t="n">
-        <v>4628910</v>
-      </c>
-      <c r="I5" s="4" t="n">
-        <v>4909315</v>
-      </c>
+        <v>4588268</v>
+      </c>
+      <c r="I5" s="5" t="n"/>
       <c r="J5" s="5" t="n"/>
       <c r="K5" s="5" t="n"/>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="2" t="n">
-        <v>1984</v>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>1985</v>
       </c>
       <c r="B6" s="4" t="n">
-        <v>310608</v>
+        <v>443160</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>1418858</v>
+        <v>1136350</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>2195047</v>
+        <v>2128333</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>3757447</v>
+        <v>2897821</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>4029929</v>
+        <v>3402672</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>4381982</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>4588268</v>
-      </c>
+        <v>3873311</v>
+      </c>
+      <c r="H6" s="5" t="n"/>
       <c r="I6" s="5" t="n"/>
       <c r="J6" s="5" t="n"/>
       <c r="K6" s="5" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="2" t="n">
-        <v>1985</v>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>1986</v>
       </c>
       <c r="B7" s="4" t="n">
-        <v>443160</v>
+        <v>396132</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>1136350</v>
+        <v>1333217</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>2128333</v>
+        <v>2180715</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>2897821</v>
+        <v>2985752</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>3402672</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>3873311</v>
-      </c>
+        <v>3691712</v>
+      </c>
+      <c r="G7" s="5" t="n"/>
       <c r="H7" s="5" t="n"/>
       <c r="I7" s="5" t="n"/>
       <c r="J7" s="5" t="n"/>
       <c r="K7" s="5" t="n"/>
     </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="n">
-        <v>1986</v>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>1987</v>
       </c>
       <c r="B8" s="4" t="n">
-        <v>396132</v>
+        <v>440832</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>1333217</v>
+        <v>1288463</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>2180715</v>
+        <v>2419861</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>2985752</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>3691712</v>
-      </c>
+        <v>3483130</v>
+      </c>
+      <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
       <c r="H8" s="5" t="n"/>
       <c r="I8" s="5" t="n"/>
       <c r="J8" s="5" t="n"/>
       <c r="K8" s="5" t="n"/>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="2" t="n">
-        <v>1987</v>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>1988</v>
       </c>
       <c r="B9" s="4" t="n">
-        <v>440832</v>
+        <v>359480</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>1288463</v>
+        <v>1421128</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>2419861</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>3483130</v>
-      </c>
+        <v>2864498</v>
+      </c>
+      <c r="E9" s="5" t="n"/>
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
       <c r="H9" s="5" t="n"/>
@@ -795,19 +787,17 @@
       <c r="J9" s="5" t="n"/>
       <c r="K9" s="5" t="n"/>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="2" t="n">
-        <v>1988</v>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>1989</v>
       </c>
       <c r="B10" s="4" t="n">
-        <v>359480</v>
+        <v>376686</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1421128</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>2864498</v>
-      </c>
+        <v>1363294</v>
+      </c>
+      <c r="D10" s="5" t="n"/>
       <c r="E10" s="5" t="n"/>
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
@@ -816,16 +806,14 @@
       <c r="J10" s="5" t="n"/>
       <c r="K10" s="5" t="n"/>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="2" t="n">
-        <v>1989</v>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>1990</v>
       </c>
       <c r="B11" s="4" t="n">
-        <v>376686</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>1363294</v>
-      </c>
+        <v>344014</v>
+      </c>
+      <c r="C11" s="5" t="n"/>
       <c r="D11" s="5" t="n"/>
       <c r="E11" s="5" t="n"/>
       <c r="F11" s="5" t="n"/>
@@ -835,27 +823,7 @@
       <c r="J11" s="5" t="n"/>
       <c r="K11" s="5" t="n"/>
     </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="2" t="n">
-        <v>1990</v>
-      </c>
-      <c r="B12" s="4" t="n">
-        <v>344014</v>
-      </c>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="5" t="n"/>
-      <c r="I12" s="5" t="n"/>
-      <c r="J12" s="5" t="n"/>
-      <c r="K12" s="5" t="n"/>
-    </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:K1"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -866,106 +834,92 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="80" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="18" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
-          <t>FORMAT A — TRIANGLE CUMULÉ</t>
+          <t>FORMAT A — TRIANGLE CUMULÉ (GenIns — Mack 1993)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="7" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>Structure :</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Colonne A : années de survenance (ex : 1981, 1982, ...)</t>
-        </is>
-      </c>
-    </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Colonnes suivantes : périodes de développement (Dev.1, Dev.2, ...)</t>
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Colonne Survenance : années d'origine (ex : 1981, 1982...)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Chaque cellule = montant CUMULÉ depuis l'origine du sinistre</t>
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Colonnes 1, 2, ... N : périodes de développement</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Cellules futures (triangle supérieur droit) : laisser VIDES — ne pas mettre 0</t>
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Chaque cellule = montant CUMULÉ depuis l'origine</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="8" t="inlineStr"/>
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Cellules futures (triangle supérieur droit) : VIDES — ne pas mettre 0</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Règles obligatoires :</t>
-        </is>
-      </c>
+      <c r="A8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Les montants doivent être croissants de gauche à droite (cumulatif)</t>
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>Règles :</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Minimum 3 années de survenance et 3 périodes de développement</t>
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Montants croissants de gauche à droite (cumulatif)</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Les montants peuvent être en euros, milliers d'euros ou millions d'euros</t>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Minimum 3 lignes × 3 colonnes</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Pas de ligne de totaux — uniquement les données</t>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Montants en euros, milliers ou millions — peu importe l'échelle</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="8" t="inlineStr"/>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t>Exemple de données GenIns (Mack 1993) inclus dans l'onglet Triangle_Paiements.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="8" t="inlineStr">
-        <is>
-          <t>Ce triangle de référence est utilisé pour la validation actuarielle.</t>
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Pas de ligne de totaux</t>
         </is>
       </c>
     </row>

</xml_diff>